<commit_message>
fix: addressing the ELSE in recode
</commit_message>
<xml_diff>
--- a/analyst/Tracy/rmonize/data_proc_elem/DPE_NAKO_TRACY.xlsx
+++ b/analyst/Tracy/rmonize/data_proc_elem/DPE_NAKO_TRACY.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\use-cases-harmonisation\analyst\Tracy\rmonize\data_proc_elem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47EC473B-3430-410D-9AFB-D26A3C9D6977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8685A59-972F-4CEB-A8AB-E348581421EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="161">
   <si>
     <t>index</t>
   </si>
@@ -501,16 +501,13 @@
     <t>a_packyears</t>
   </si>
   <si>
-    <t>recode(1= 1; 2 = 0;ELSE=NA;)</t>
-  </si>
-  <si>
-    <t>recode(1= 1; 2 = 0;ELSE=NA)</t>
-  </si>
-  <si>
     <t>a_diab</t>
   </si>
   <si>
     <t>undetermined</t>
+  </si>
+  <si>
+    <t>recode(1= 1; 2 = 0;)</t>
   </si>
 </sst>
 </file>
@@ -1140,17 +1137,17 @@
         <v>13</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I8" s="7"/>
       <c r="J8" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -1190,17 +1187,17 @@
         <v>18</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I10" s="7"/>
       <c r="J10" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1240,17 +1237,17 @@
         <v>18</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I12" s="7"/>
       <c r="J12" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K12" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -1290,17 +1287,17 @@
         <v>13</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I14" s="7"/>
       <c r="J14" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K14" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -1314,17 +1311,17 @@
         <v>13</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I15" s="7"/>
       <c r="J15" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1344,7 +1341,7 @@
         <v>150</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="J16" s="5" t="s">
         <v>135</v>
@@ -1436,7 +1433,7 @@
         <v>13</v>
       </c>
       <c r="F20" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G20" s="4" t="s">
         <v>138</v>
@@ -1468,7 +1465,7 @@
         <v>150</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="J21" s="5" t="s">
         <v>135</v>
@@ -1489,17 +1486,17 @@
       </c>
       <c r="F22" s="8"/>
       <c r="G22" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I22" s="7"/>
       <c r="J22" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K22" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.25">
@@ -1519,7 +1516,7 @@
         <v>150</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="J23" s="5" t="s">
         <v>135</v>
@@ -1539,17 +1536,17 @@
         <v>13</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I24" s="7"/>
       <c r="J24" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K24" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.25">
@@ -1563,17 +1560,17 @@
         <v>13</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I25" s="7"/>
       <c r="J25" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K25" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="26" spans="2:11" x14ac:dyDescent="0.25">
@@ -1587,17 +1584,17 @@
         <v>13</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I26" s="7"/>
       <c r="J26" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K26" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.25">
@@ -1680,17 +1677,17 @@
         <v>13</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I30" s="7"/>
       <c r="J30" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K30" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="31" spans="2:11" x14ac:dyDescent="0.25">
@@ -1704,17 +1701,17 @@
         <v>13</v>
       </c>
       <c r="G31" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I31" s="7"/>
       <c r="J31" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K31" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="32" spans="2:11" x14ac:dyDescent="0.25">
@@ -2281,17 +2278,17 @@
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>
       <c r="G54" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H54" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I54" s="7"/>
       <c r="J54" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K54" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="55" spans="2:11" s="12" customFormat="1" x14ac:dyDescent="0.25">
@@ -2307,17 +2304,17 @@
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>
       <c r="G55" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I55" s="7"/>
       <c r="J55" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K55" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="56" spans="2:11" x14ac:dyDescent="0.25">
@@ -2333,17 +2330,17 @@
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
       <c r="G56" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H56" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I56" s="7"/>
       <c r="J56" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K56" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="57" spans="2:11" s="12" customFormat="1" x14ac:dyDescent="0.25">
@@ -2359,17 +2356,17 @@
       <c r="E57" s="2"/>
       <c r="F57" s="2"/>
       <c r="G57" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I57" s="7"/>
       <c r="J57" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K57" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="58" spans="2:11" s="12" customFormat="1" x14ac:dyDescent="0.25">
@@ -2385,17 +2382,17 @@
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
       <c r="G58" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H58" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I58" s="7"/>
       <c r="J58" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K58" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="59" spans="2:11" s="12" customFormat="1" x14ac:dyDescent="0.25">
@@ -2411,17 +2408,17 @@
       <c r="E59" s="2"/>
       <c r="F59" s="2"/>
       <c r="G59" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I59" s="7"/>
       <c r="J59" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K59" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="60" spans="2:11" s="12" customFormat="1" x14ac:dyDescent="0.25">
@@ -2437,17 +2434,17 @@
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
       <c r="G60" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H60" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I60" s="7"/>
       <c r="J60" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K60" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="61" spans="2:11" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -2463,16 +2460,16 @@
       <c r="E61" s="2"/>
       <c r="F61" s="2"/>
       <c r="G61" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="J61" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K61" s="7" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>